<commit_message>
Arreglado reporte req. hotel
</commit_message>
<xml_diff>
--- a/ejemplo_carga_masiva.xlsx
+++ b/ejemplo_carga_masiva.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="ON" sheetId="1" state="visible" r:id="rId3"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2440" uniqueCount="599">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2440" uniqueCount="600">
   <si>
     <t xml:space="preserve">Owner</t>
   </si>
@@ -1773,6 +1773,9 @@
   </si>
   <si>
     <t xml:space="preserve">OKUSA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PUQ Almuerzo</t>
   </si>
   <si>
     <t xml:space="preserve">ATO SCL</t>
@@ -16261,13 +16264,13 @@
         <v>583</v>
       </c>
       <c r="BM3" s="32" t="s">
-        <v>251</v>
+        <v>584</v>
       </c>
       <c r="BN3" s="49" t="n">
-        <v>45557</v>
+        <v>45558</v>
       </c>
       <c r="BO3" s="49" t="n">
-        <v>45557</v>
+        <v>45559</v>
       </c>
       <c r="BP3" s="32" t="s">
         <v>583</v>
@@ -16276,22 +16279,22 @@
         <v>251</v>
       </c>
       <c r="BR3" s="49" t="n">
-        <v>45557</v>
+        <v>45559</v>
       </c>
       <c r="BS3" s="49" t="n">
-        <v>45557</v>
+        <v>45560</v>
       </c>
       <c r="BT3" s="32" t="s">
         <v>583</v>
       </c>
       <c r="BU3" s="32" t="s">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="BV3" s="32" t="s">
         <v>128</v>
       </c>
       <c r="BW3" s="32" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="BX3" s="49" t="n">
         <v>45557</v>
@@ -16302,10 +16305,10 @@
     </row>
     <row r="4" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="32" t="s">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="B4" s="32" t="s">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="C4" s="33" t="n">
         <v>45918</v>
@@ -16317,33 +16320,33 @@
         <v>45918</v>
       </c>
       <c r="F4" s="32" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="G4" s="32" t="s">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="H4" s="32"/>
       <c r="I4" s="32"/>
       <c r="J4" s="32" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="K4" s="32" t="s">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="L4" s="32" t="s">
         <v>95</v>
       </c>
       <c r="M4" s="32" t="s">
-        <v>592</v>
+        <v>593</v>
       </c>
       <c r="N4" s="32" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="O4" s="32" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="P4" s="33" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="Q4" s="32"/>
       <c r="R4" s="32"/>
@@ -16356,7 +16359,7 @@
         <v>45611</v>
       </c>
       <c r="W4" s="32" t="s">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="X4" s="32" t="s">
         <v>573</v>
@@ -16365,7 +16368,7 @@
         <v>45558</v>
       </c>
       <c r="Z4" s="32" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="AA4" s="32"/>
       <c r="AB4" s="32"/>
@@ -16426,7 +16429,7 @@
       <c r="BU4" s="32"/>
       <c r="BV4" s="32"/>
       <c r="BW4" s="32" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="BX4" s="32"/>
       <c r="BY4" s="32" t="s">

</xml_diff>